<commit_message>
fix: update notification logic in multiple controllers to send notifications to specific users and adjust UI layout in warming up genset view
</commit_message>
<xml_diff>
--- a/public/assets/templates/operasional/genset.xlsx
+++ b/public/assets/templates/operasional/genset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\operasional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E9F49C-C9B8-46C7-8C34-60A8B5B7AA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E137817C-5166-4B19-89E0-F87AC56C9356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{9899F60B-4AD3-4F48-B76C-CA7BD2003EFF}"/>
   </bookViews>
@@ -529,7 +529,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -576,97 +576,109 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1042,97 +1054,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickTop="1">
-      <c r="A1" s="30"/>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="34" t="s">
+      <c r="A1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="40" t="s">
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="41"/>
+      <c r="K1" s="29"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="32"/>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="43"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="31"/>
     </row>
     <row r="3" spans="1:11" ht="20.5" thickBot="1">
-      <c r="A3" s="32"/>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="44" t="s">
+      <c r="A3" s="20"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="45"/>
-      <c r="H3" s="45"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="42"/>
-      <c r="K3" s="43"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="31"/>
     </row>
     <row r="4" spans="1:11" ht="34" customHeight="1" thickTop="1">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="24" t="s">
+      <c r="K4" s="39" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1">
-      <c r="A5" s="27"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="25"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="40"/>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1"/>
@@ -1553,94 +1565,94 @@
       <c r="K37" s="12"/>
     </row>
     <row r="38" spans="1:11" ht="15" thickTop="1">
-      <c r="A38" s="16" t="s">
+      <c r="A38" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
+      <c r="B38" s="42"/>
+      <c r="C38" s="42"/>
       <c r="D38" s="13"/>
-      <c r="E38" s="17" t="s">
+      <c r="E38" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
       <c r="H38" s="13"/>
-      <c r="I38" s="17" t="s">
+      <c r="I38" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="J38" s="17"/>
-      <c r="K38" s="18"/>
+      <c r="J38" s="42"/>
+      <c r="K38" s="43"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="9"/>
-      <c r="B39" s="10"/>
-      <c r="C39" s="11"/>
+      <c r="A39" s="47"/>
+      <c r="B39" s="48"/>
+      <c r="C39" s="48"/>
       <c r="D39" s="11"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
       <c r="H39" s="11"/>
-      <c r="I39" s="10"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="12"/>
+      <c r="I39" s="49"/>
+      <c r="J39" s="49"/>
+      <c r="K39" s="50"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="9"/>
-      <c r="B40" s="10"/>
-      <c r="C40" s="11"/>
+      <c r="A40" s="47"/>
+      <c r="B40" s="48"/>
+      <c r="C40" s="48"/>
       <c r="D40" s="11"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
+      <c r="E40" s="49"/>
+      <c r="F40" s="49"/>
+      <c r="G40" s="49"/>
       <c r="H40" s="11"/>
-      <c r="I40" s="10"/>
-      <c r="J40" s="11"/>
-      <c r="K40" s="12"/>
+      <c r="I40" s="49"/>
+      <c r="J40" s="49"/>
+      <c r="K40" s="50"/>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="9"/>
-      <c r="B41" s="10"/>
-      <c r="C41" s="11"/>
+      <c r="A41" s="47"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
       <c r="D41" s="11"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
+      <c r="G41" s="49"/>
       <c r="H41" s="11"/>
-      <c r="I41" s="10"/>
-      <c r="J41" s="11"/>
-      <c r="K41" s="12"/>
+      <c r="I41" s="49"/>
+      <c r="J41" s="49"/>
+      <c r="K41" s="50"/>
     </row>
     <row r="42" spans="1:11">
-      <c r="A42" s="9"/>
-      <c r="B42" s="10"/>
-      <c r="C42" s="11"/>
+      <c r="A42" s="47"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
       <c r="D42" s="11"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49"/>
       <c r="H42" s="11"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="12"/>
+      <c r="I42" s="49"/>
+      <c r="J42" s="49"/>
+      <c r="K42" s="50"/>
     </row>
     <row r="43" spans="1:11" ht="15" thickBot="1">
-      <c r="A43" s="19" t="s">
+      <c r="A43" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
+      <c r="B43" s="45"/>
+      <c r="C43" s="45"/>
       <c r="D43" s="14"/>
-      <c r="E43" s="20" t="s">
+      <c r="E43" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="F43" s="20"/>
-      <c r="G43" s="20"/>
+      <c r="F43" s="45"/>
+      <c r="G43" s="45"/>
       <c r="H43" s="14"/>
-      <c r="I43" s="20" t="s">
+      <c r="I43" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="J43" s="20"/>
-      <c r="K43" s="21"/>
+      <c r="J43" s="45"/>
+      <c r="K43" s="46"/>
     </row>
     <row r="44" spans="1:11" ht="15" thickTop="1">
       <c r="A44" s="10"/>
@@ -1657,7 +1669,16 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="24">
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="I38:K38"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="A39:C42"/>
+    <mergeCell ref="E39:G42"/>
+    <mergeCell ref="I39:K42"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="A1:C3"/>
@@ -1673,12 +1694,6 @@
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="J4:J5"/>
     <mergeCell ref="K4:K5"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="I43:K43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add username and time submit to export
</commit_message>
<xml_diff>
--- a/public/assets/templates/operasional/genset.xlsx
+++ b/public/assets/templates/operasional/genset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\operasional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E137817C-5166-4B19-89E0-F87AC56C9356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B73AE4-D508-424A-9043-DC153495DB67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{9899F60B-4AD3-4F48-B76C-CA7BD2003EFF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>PT BUMI ALAM SEGAR</t>
   </si>
@@ -78,26 +78,17 @@
     <t>SPV Engineering</t>
   </si>
   <si>
-    <t>(                                      )</t>
-  </si>
-  <si>
-    <t>(                                          )</t>
-  </si>
-  <si>
     <t>Staff Engineering</t>
   </si>
   <si>
     <t>Pelaksana</t>
-  </si>
-  <si>
-    <t>(                                           )</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,6 +128,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -146,7 +167,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -484,23 +505,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
+      <left style="thin">
         <color auto="1"/>
       </left>
       <right/>
-      <top style="double">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="double">
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -508,19 +520,23 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="double">
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="double">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="double">
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -529,7 +545,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -567,15 +583,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -651,36 +658,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1044,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E30EF17F-5FFC-4A29-B061-FAC82A185028}">
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1054,97 +1052,97 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickTop="1">
-      <c r="A1" s="18"/>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="22" t="s">
+      <c r="A1" s="15"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="28" t="s">
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="29"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="20"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="31"/>
+      <c r="A2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="28"/>
     </row>
     <row r="3" spans="1:11" ht="20.5" thickBot="1">
-      <c r="A3" s="20"/>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="32" t="s">
+      <c r="A3" s="17"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="31"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="28"/>
     </row>
     <row r="4" spans="1:11" ht="34" customHeight="1" thickTop="1">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="K4" s="39" t="s">
+      <c r="K4" s="36" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="30" customHeight="1">
-      <c r="A5" s="36"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="40"/>
+      <c r="A5" s="33"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="37"/>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="1"/>
@@ -1551,7 +1549,7 @@
       <c r="J36" s="7"/>
       <c r="K36" s="8"/>
     </row>
-    <row r="37" spans="1:11" ht="15.5" thickTop="1" thickBot="1">
+    <row r="37" spans="1:11" ht="15" thickTop="1">
       <c r="A37" s="9"/>
       <c r="B37" s="10"/>
       <c r="C37" s="11"/>
@@ -1564,121 +1562,124 @@
       <c r="J37" s="11"/>
       <c r="K37" s="12"/>
     </row>
-    <row r="38" spans="1:11" ht="15" thickTop="1">
-      <c r="A38" s="41" t="s">
-        <v>20</v>
-      </c>
-      <c r="B38" s="42"/>
-      <c r="C38" s="42"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="42" t="s">
-        <v>19</v>
-      </c>
-      <c r="F38" s="42"/>
-      <c r="G38" s="42"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="42" t="s">
+    <row r="38" spans="1:11" s="44" customFormat="1">
+      <c r="A38" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="E38" s="40"/>
+      <c r="F38" s="40"/>
+      <c r="G38" s="41"/>
+      <c r="H38" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="J38" s="42"/>
-      <c r="K38" s="43"/>
-    </row>
-    <row r="39" spans="1:11">
-      <c r="A39" s="47"/>
-      <c r="B39" s="48"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="49"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="49"/>
-      <c r="J39" s="49"/>
-      <c r="K39" s="50"/>
-    </row>
-    <row r="40" spans="1:11">
-      <c r="A40" s="47"/>
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="49"/>
-      <c r="F40" s="49"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="49"/>
-      <c r="J40" s="49"/>
-      <c r="K40" s="50"/>
-    </row>
-    <row r="41" spans="1:11">
-      <c r="A41" s="47"/>
-      <c r="B41" s="48"/>
-      <c r="C41" s="48"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="49"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="49"/>
-      <c r="J41" s="49"/>
-      <c r="K41" s="50"/>
-    </row>
-    <row r="42" spans="1:11">
-      <c r="A42" s="47"/>
-      <c r="B42" s="48"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="49"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="49"/>
-      <c r="J42" s="49"/>
-      <c r="K42" s="50"/>
-    </row>
-    <row r="43" spans="1:11" ht="15" thickBot="1">
-      <c r="A43" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="B43" s="45"/>
-      <c r="C43" s="45"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="45" t="s">
-        <v>18</v>
-      </c>
-      <c r="F43" s="45"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="J43" s="45"/>
-      <c r="K43" s="46"/>
-    </row>
-    <row r="44" spans="1:11" ht="15" thickTop="1">
-      <c r="A44" s="10"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="J44" s="15"/>
-      <c r="K44" s="15" t="s">
+      <c r="I38" s="40"/>
+      <c r="J38" s="40"/>
+      <c r="K38" s="41"/>
+    </row>
+    <row r="39" spans="1:11" s="44" customFormat="1">
+      <c r="A39" s="18"/>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+    </row>
+    <row r="40" spans="1:11" s="44" customFormat="1">
+      <c r="A40" s="18"/>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+    </row>
+    <row r="41" spans="1:11" s="44" customFormat="1">
+      <c r="A41" s="18"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="18"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+    </row>
+    <row r="42" spans="1:11" s="44" customFormat="1">
+      <c r="A42" s="18"/>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="18"/>
+      <c r="J42" s="18"/>
+      <c r="K42" s="18"/>
+    </row>
+    <row r="43" spans="1:11" s="45" customFormat="1">
+      <c r="A43" s="42"/>
+      <c r="B43" s="42"/>
+      <c r="C43" s="42"/>
+      <c r="D43" s="42"/>
+      <c r="E43" s="42"/>
+      <c r="F43" s="42"/>
+      <c r="G43" s="42"/>
+      <c r="H43" s="42"/>
+      <c r="I43" s="42"/>
+      <c r="J43" s="42"/>
+      <c r="K43" s="42"/>
+    </row>
+    <row r="44" spans="1:11" s="46" customFormat="1">
+      <c r="A44" s="43"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="43"/>
+      <c r="D44" s="43"/>
+      <c r="E44" s="43"/>
+      <c r="F44" s="43"/>
+      <c r="G44" s="43"/>
+      <c r="H44" s="43"/>
+      <c r="I44" s="43"/>
+      <c r="J44" s="43"/>
+      <c r="K44" s="43"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="A45" s="10"/>
+      <c r="B45" s="11"/>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="11"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11"/>
+      <c r="H45" s="11"/>
+      <c r="J45" s="38"/>
+      <c r="K45" s="38" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="I38:K38"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="A39:C42"/>
-    <mergeCell ref="E39:G42"/>
-    <mergeCell ref="I39:K42"/>
+  <mergeCells count="27">
+    <mergeCell ref="D44:G44"/>
+    <mergeCell ref="H43:K43"/>
+    <mergeCell ref="H44:K44"/>
+    <mergeCell ref="D38:G38"/>
+    <mergeCell ref="H38:K38"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="A1:C3"/>
@@ -1694,8 +1695,16 @@
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="J4:J5"/>
     <mergeCell ref="K4:K5"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A39:C42"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="H39:K42"/>
+    <mergeCell ref="D39:G42"/>
+    <mergeCell ref="D43:G43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>